<commit_message>
Resumo de atividade — 8 de setembro de 2026
</commit_message>
<xml_diff>
--- a/Resumo_atividade/Resumo-survey_os_20260908.xlsx
+++ b/Resumo_atividade/Resumo-survey_os_20260908.xlsx
@@ -91,6 +91,12 @@
     <t>Ivan</t>
   </si>
   <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>Prudentópolis</t>
+  </si>
+  <si>
     <t>-25.221782, -51.000775</t>
   </si>
   <si>
@@ -98,12 +104,6 @@
   </si>
   <si>
     <t>OS-2026-0121</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>Prudentópolis</t>
   </si>
   <si>
     <t>Avenida São João</t>
@@ -1667,10 +1667,10 @@
         <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
         <v>22</v>
@@ -1679,10 +1679,10 @@
         <v>22</v>
       </c>
       <c r="I3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K3" t="s">
         <v>25</v>
@@ -1696,7 +1696,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
@@ -1708,10 +1708,10 @@
         <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
         <v>22</v>
@@ -1723,7 +1723,7 @@
         <v>32</v>
       </c>
       <c r="J4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K4" t="s">
         <v>25</v>
@@ -1749,10 +1749,10 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
         <v>22</v>
@@ -1764,7 +1764,7 @@
         <v>36</v>
       </c>
       <c r="J5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K5" t="s">
         <v>25</v>
@@ -1790,10 +1790,10 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
         <v>22</v>
@@ -1805,7 +1805,7 @@
         <v>38</v>
       </c>
       <c r="J6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K6" t="s">
         <v>25</v>
@@ -1831,10 +1831,10 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
         <v>22</v>
@@ -1846,7 +1846,7 @@
         <v>40</v>
       </c>
       <c r="J7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K7" t="s">
         <v>25</v>
@@ -1872,10 +1872,10 @@
         <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
         <v>22</v>
@@ -1887,7 +1887,7 @@
         <v>42</v>
       </c>
       <c r="J8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K8" t="s">
         <v>25</v>
@@ -1913,10 +1913,10 @@
         <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
         <v>22</v>
@@ -1928,7 +1928,7 @@
         <v>45</v>
       </c>
       <c r="J9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K9" t="s">
         <v>25</v>
@@ -1954,10 +1954,10 @@
         <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G10" t="s">
         <v>22</v>
@@ -1969,7 +1969,7 @@
         <v>47</v>
       </c>
       <c r="J10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K10" t="s">
         <v>25</v>
@@ -1995,7 +1995,7 @@
         <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
         <v>51</v>
@@ -2010,7 +2010,7 @@
         <v>53</v>
       </c>
       <c r="J11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K11" t="s">
         <v>50</v>
@@ -2036,10 +2036,10 @@
         <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G12" t="s">
         <v>22</v>
@@ -2051,7 +2051,7 @@
         <v>55</v>
       </c>
       <c r="J12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K12" t="s">
         <v>25</v>
@@ -2077,10 +2077,10 @@
         <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G13" t="s">
         <v>22</v>
@@ -2092,7 +2092,7 @@
         <v>57</v>
       </c>
       <c r="J13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K13" t="s">
         <v>25</v>
@@ -2118,10 +2118,10 @@
         <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G14" t="s">
         <v>22</v>
@@ -2133,7 +2133,7 @@
         <v>59</v>
       </c>
       <c r="J14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K14" t="s">
         <v>25</v>
@@ -2159,10 +2159,10 @@
         <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G15" t="s">
         <v>22</v>
@@ -2174,7 +2174,7 @@
         <v>61</v>
       </c>
       <c r="J15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K15" t="s">
         <v>25</v>
@@ -2200,10 +2200,10 @@
         <v>25</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G16" t="s">
         <v>22</v>
@@ -2215,7 +2215,7 @@
         <v>61</v>
       </c>
       <c r="J16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K16" t="s">
         <v>25</v>
@@ -2364,10 +2364,10 @@
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G20" t="s">
         <v>22</v>
@@ -2379,7 +2379,7 @@
         <v>83</v>
       </c>
       <c r="J20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K20" t="s">
         <v>25</v>
@@ -2405,10 +2405,10 @@
         <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G21" t="s">
         <v>22</v>
@@ -2420,7 +2420,7 @@
         <v>86</v>
       </c>
       <c r="J21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K21" t="s">
         <v>25</v>
@@ -2446,10 +2446,10 @@
         <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G22" t="s">
         <v>22</v>
@@ -2461,7 +2461,7 @@
         <v>86</v>
       </c>
       <c r="J22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K22" t="s">
         <v>25</v>
@@ -2487,10 +2487,10 @@
         <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G23" t="s">
         <v>22</v>
@@ -2502,7 +2502,7 @@
         <v>90</v>
       </c>
       <c r="J23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K23" t="s">
         <v>25</v>
@@ -2528,10 +2528,10 @@
         <v>25</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F24" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G24" t="s">
         <v>22</v>
@@ -2543,7 +2543,7 @@
         <v>93</v>
       </c>
       <c r="J24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K24" t="s">
         <v>25</v>
@@ -2569,10 +2569,10 @@
         <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G25" t="s">
         <v>22</v>
@@ -2584,7 +2584,7 @@
         <v>95</v>
       </c>
       <c r="J25" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K25" t="s">
         <v>25</v>
@@ -2610,10 +2610,10 @@
         <v>97</v>
       </c>
       <c r="E26" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G26" t="s">
         <v>22</v>
@@ -2625,7 +2625,7 @@
         <v>99</v>
       </c>
       <c r="J26" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K26" t="s">
         <v>97</v>
@@ -2651,10 +2651,10 @@
         <v>97</v>
       </c>
       <c r="E27" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G27" t="s">
         <v>22</v>
@@ -2666,7 +2666,7 @@
         <v>101</v>
       </c>
       <c r="J27" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K27" t="s">
         <v>97</v>
@@ -2692,7 +2692,7 @@
         <v>104</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F28" t="s">
         <v>105</v>
@@ -2707,7 +2707,7 @@
         <v>108</v>
       </c>
       <c r="J28" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K28" t="s">
         <v>109</v>
@@ -2733,7 +2733,7 @@
         <v>104</v>
       </c>
       <c r="E29" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F29" t="s">
         <v>105</v>
@@ -2748,7 +2748,7 @@
         <v>22</v>
       </c>
       <c r="J29" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K29" t="s">
         <v>109</v>
@@ -2774,10 +2774,10 @@
         <v>97</v>
       </c>
       <c r="E30" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F30" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G30" t="s">
         <v>22</v>
@@ -2789,7 +2789,7 @@
         <v>115</v>
       </c>
       <c r="J30" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K30" t="s">
         <v>97</v>
@@ -2815,10 +2815,10 @@
         <v>97</v>
       </c>
       <c r="E31" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F31" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G31" t="s">
         <v>22</v>
@@ -2830,7 +2830,7 @@
         <v>117</v>
       </c>
       <c r="J31" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K31" t="s">
         <v>97</v>
@@ -2856,10 +2856,10 @@
         <v>97</v>
       </c>
       <c r="E32" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G32" t="s">
         <v>22</v>
@@ -2871,7 +2871,7 @@
         <v>119</v>
       </c>
       <c r="J32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K32" t="s">
         <v>97</v>
@@ -2897,10 +2897,10 @@
         <v>97</v>
       </c>
       <c r="E33" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G33" t="s">
         <v>22</v>
@@ -2912,7 +2912,7 @@
         <v>122</v>
       </c>
       <c r="J33" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K33" t="s">
         <v>97</v>
@@ -2938,7 +2938,7 @@
         <v>124</v>
       </c>
       <c r="E34" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F34" t="s">
         <v>125</v>
@@ -2953,7 +2953,7 @@
         <v>128</v>
       </c>
       <c r="J34" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K34" t="s">
         <v>124</v>
@@ -2979,10 +2979,10 @@
         <v>97</v>
       </c>
       <c r="E35" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G35" t="s">
         <v>22</v>
@@ -2994,7 +2994,7 @@
         <v>130</v>
       </c>
       <c r="J35" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K35" t="s">
         <v>97</v>
@@ -3020,10 +3020,10 @@
         <v>97</v>
       </c>
       <c r="E36" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F36" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G36" t="s">
         <v>22</v>
@@ -3035,7 +3035,7 @@
         <v>132</v>
       </c>
       <c r="J36" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K36" t="s">
         <v>97</v>
@@ -3061,7 +3061,7 @@
         <v>134</v>
       </c>
       <c r="E37" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F37" t="s">
         <v>51</v>
@@ -3076,7 +3076,7 @@
         <v>137</v>
       </c>
       <c r="J37" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K37" t="s">
         <v>50</v>
@@ -3102,7 +3102,7 @@
         <v>139</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F38" t="s">
         <v>125</v>
@@ -3117,7 +3117,7 @@
         <v>142</v>
       </c>
       <c r="J38" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K38" t="s">
         <v>124</v>
@@ -3143,7 +3143,7 @@
         <v>144</v>
       </c>
       <c r="E39" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F39" t="s">
         <v>145</v>
@@ -3158,7 +3158,7 @@
         <v>22</v>
       </c>
       <c r="J39" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K39" t="s">
         <v>124</v>
@@ -3266,7 +3266,7 @@
         <v>165</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F42" t="s">
         <v>166</v>
@@ -3348,7 +3348,7 @@
         <v>165</v>
       </c>
       <c r="E44" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F44" t="s">
         <v>178</v>
@@ -3363,7 +3363,7 @@
         <v>180</v>
       </c>
       <c r="J44" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K44" t="s">
         <v>181</v>
@@ -3389,7 +3389,7 @@
         <v>165</v>
       </c>
       <c r="E45" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F45" t="s">
         <v>183</v>
@@ -3404,7 +3404,7 @@
         <v>22</v>
       </c>
       <c r="J45" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K45" t="s">
         <v>109</v>
@@ -3471,7 +3471,7 @@
         <v>191</v>
       </c>
       <c r="E47" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F47" t="s">
         <v>192</v>
@@ -3486,7 +3486,7 @@
         <v>195</v>
       </c>
       <c r="J47" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K47" t="s">
         <v>196</v>
@@ -3512,7 +3512,7 @@
         <v>50</v>
       </c>
       <c r="E48" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F48" t="s">
         <v>51</v>
@@ -3527,7 +3527,7 @@
         <v>198</v>
       </c>
       <c r="J48" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K48" t="s">
         <v>50</v>
@@ -3594,7 +3594,7 @@
         <v>50</v>
       </c>
       <c r="E50" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F50" t="s">
         <v>51</v>
@@ -3609,7 +3609,7 @@
         <v>53</v>
       </c>
       <c r="J50" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K50" t="s">
         <v>50</v>
@@ -3840,7 +3840,7 @@
         <v>144</v>
       </c>
       <c r="E56" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F56" t="s">
         <v>145</v>
@@ -3855,7 +3855,7 @@
         <v>22</v>
       </c>
       <c r="J56" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K56" t="s">
         <v>124</v>
@@ -3881,7 +3881,7 @@
         <v>226</v>
       </c>
       <c r="E57" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F57" t="s">
         <v>51</v>
@@ -3896,7 +3896,7 @@
         <v>227</v>
       </c>
       <c r="J57" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K57" t="s">
         <v>50</v>
@@ -3922,7 +3922,7 @@
         <v>165</v>
       </c>
       <c r="E58" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F58" t="s">
         <v>229</v>
@@ -3937,7 +3937,7 @@
         <v>231</v>
       </c>
       <c r="J58" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K58" t="s">
         <v>181</v>
@@ -3963,7 +3963,7 @@
         <v>233</v>
       </c>
       <c r="E59" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F59" t="s">
         <v>234</v>
@@ -3978,7 +3978,7 @@
         <v>236</v>
       </c>
       <c r="J59" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K59" t="s">
         <v>181</v>
@@ -4086,7 +4086,7 @@
         <v>247</v>
       </c>
       <c r="E62" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F62" t="s">
         <v>192</v>
@@ -4127,7 +4127,7 @@
         <v>252</v>
       </c>
       <c r="E63" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F63" t="s">
         <v>253</v>
@@ -4142,7 +4142,7 @@
         <v>256</v>
       </c>
       <c r="J63" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K63" t="s">
         <v>50</v>
@@ -4168,7 +4168,7 @@
         <v>191</v>
       </c>
       <c r="E64" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F64" t="s">
         <v>258</v>
@@ -4209,7 +4209,7 @@
         <v>233</v>
       </c>
       <c r="E65" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F65" t="s">
         <v>234</v>
@@ -4224,7 +4224,7 @@
         <v>264</v>
       </c>
       <c r="J65" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K65" t="s">
         <v>181</v>
@@ -4291,7 +4291,7 @@
         <v>139</v>
       </c>
       <c r="E67" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F67" t="s">
         <v>125</v>
@@ -4414,7 +4414,7 @@
         <v>233</v>
       </c>
       <c r="E70" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F70" t="s">
         <v>234</v>
@@ -4429,7 +4429,7 @@
         <v>286</v>
       </c>
       <c r="J70" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K70" t="s">
         <v>181</v>
@@ -4537,7 +4537,7 @@
         <v>296</v>
       </c>
       <c r="E73" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F73" t="s">
         <v>51</v>
@@ -4552,7 +4552,7 @@
         <v>298</v>
       </c>
       <c r="J73" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K73" t="s">
         <v>50</v>
@@ -4701,7 +4701,7 @@
         <v>313</v>
       </c>
       <c r="E77" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F77" t="s">
         <v>192</v>
@@ -4742,7 +4742,7 @@
         <v>318</v>
       </c>
       <c r="E78" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F78" t="s">
         <v>178</v>
@@ -4757,7 +4757,7 @@
         <v>321</v>
       </c>
       <c r="J78" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K78" t="s">
         <v>181</v>
@@ -4865,7 +4865,7 @@
         <v>331</v>
       </c>
       <c r="E81" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F81" t="s">
         <v>332</v>
@@ -4880,7 +4880,7 @@
         <v>335</v>
       </c>
       <c r="J81" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K81" t="s">
         <v>50</v>
@@ -4906,7 +4906,7 @@
         <v>313</v>
       </c>
       <c r="E82" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F82" t="s">
         <v>192</v>
@@ -4947,7 +4947,7 @@
         <v>341</v>
       </c>
       <c r="E83" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F83" t="s">
         <v>192</v>
@@ -5152,7 +5152,7 @@
         <v>191</v>
       </c>
       <c r="E88" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F88" t="s">
         <v>258</v>
@@ -5167,7 +5167,7 @@
         <v>366</v>
       </c>
       <c r="J88" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K88" t="s">
         <v>196</v>
@@ -5193,7 +5193,7 @@
         <v>313</v>
       </c>
       <c r="E89" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F89" t="s">
         <v>192</v>
@@ -5208,7 +5208,7 @@
         <v>370</v>
       </c>
       <c r="J89" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K89" t="s">
         <v>196</v>
@@ -5234,7 +5234,7 @@
         <v>233</v>
       </c>
       <c r="E90" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F90" t="s">
         <v>234</v>
@@ -5249,7 +5249,7 @@
         <v>374</v>
       </c>
       <c r="J90" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K90" t="s">
         <v>181</v>

</xml_diff>